<commit_message>
report: 2026-10-27 + skill 经验更新(A15-A18)
</commit_message>
<xml_diff>
--- a/股票预测/股票预测总表.xlsx
+++ b/股票预测/股票预测总表.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -104,7 +107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +140,12 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -217,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyStockPrediction" displayName="DailyStockPrediction" ref="A1:M3" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyStockPrediction" displayName="DailyStockPrediction" ref="A1:M4" headerRowCount="1">
   <autoFilter ref="A1:M3"/>
   <tableColumns count="13">
     <tableColumn id="1" name="序号"/>
@@ -527,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -709,7 +718,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>10-23：开盘2/4；收盘0/4；板块和个股部分准确；综合1/6</t>
+          <t>10-26：开盘1/4；收盘2/4；板块与个股部分准确；综合2/6</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -737,9 +746,9 @@
           <t>202610/2026-10-26_3.jpg</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>待验证</t>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>已验证：开盘1/4；收盘2/4；板块与个股部分准确；综合2/6</t>
         </is>
       </c>
       <c r="N3" s="11" t="inlineStr">
@@ -750,6 +759,66 @@
 恒生科技：平开至小幅低开 3835~3875；收盘中性偏弱 3824~3862；全天 3810~3865；置信度 中低。
 首要变量：南向连续净卖出、腾讯/小米带动、3900压力、美联储议息、中概与汇率。
 （参考昨收按今日预估收盘≈上证3690/恒科3860；区间遵循≤1%/≤1.5%规则；今日截至14:30实际：上证≈3690平盘、恒科≈3872微跌）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>平开略偏强 3696~3712</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>小幅高开 2640~2658</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>平开略偏强 23200~23300</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>小幅高开 3860~3892</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>202610/2026-10-27.md</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>202610/2026-10-27_1.jpg</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>202610/2026-10-27_2.jpg</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>202610/2026-10-27_3.jpg</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>【待填·收盘前 14:30 预测下一开盘日 2026-10-28】今晨预测已锁定：上证平开略偏强3696~3712、创业板小幅高开2640~2658、恒指23200~23300、恒科3860~3892。今日收盘前需补记对10-28的开盘/收盘区间预判（区间≤1%/≤1.5%）。</t>
         </is>
       </c>
     </row>
@@ -764,10 +833,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
report: 2026-10-27 收盘前预测下一交易日(2026-10-28 上证/恒科)
</commit_message>
<xml_diff>
--- a/股票预测/股票预测总表.xlsx
+++ b/股票预测/股票预测总表.xlsx
@@ -818,7 +818,12 @@
       </c>
       <c r="N4" s="13" t="inlineStr">
         <is>
-          <t>【待填·收盘前 14:30 预测下一开盘日 2026-10-28】今晨预测已锁定：上证平开略偏强3696~3712、创业板小幅高开2640~2658、恒指23200~23300、恒科3860~3892。今日收盘前需补记对10-28的开盘/收盘区间预判（区间≤1%/≤1.5%）。</t>
+          <t>【收盘前预测·下一开盘日 2026-10-28】
+上证指数：平开略偏弱 3670~3690；收盘中性偏弱 3668~3696；全天 3662~3700；置信度 中。
+首要变量：美联储10/27-28议息（10/28凌晨出结果）、3675附近承接、3700~3720压力、量能、五中全会会期维稳。
+恒生科技：平开至小幅低开 3802~3840；收盘中性偏弱 3800~3838；全天 3792~3846；置信度 中。
+首要变量：南向连续净卖出、美股科技/费半传导、3900压力、美联储议息与美债汇率、美方限投细则压制。
+（基准按今日预估收盘≈上证3680/恒科3820；区间遵循≤1%/≤1.5%规则；今日截至14:25实际：上证≈3677.56(-0.54%)、恒科≈3819.06(-1.00%)，均偏弱）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
report: 2026-10-28 收盘前预测下一交易日(2026-10-29 上证/恒科)
</commit_message>
<xml_diff>
--- a/股票预测/股票预测总表.xlsx
+++ b/股票预测/股票预测总表.xlsx
@@ -107,7 +107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -149,6 +149,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -862,7 +865,11 @@
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>今日（10-28）弱修复反弹：创业板+3.1%/上证+0.9%/恒科+0.9%；美联储10/29凌晨决议（预期按兵不动）；五中全会29日闭幕、维稳尾段；“外部映射失效”模式仍在、前两日放量杀跌筹码未清；南向连续净卖出；量能决定反弹能否延续</t>
+        </is>
+      </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
           <t>202610/2026-10-28.md</t>
@@ -891,9 +898,15 @@
       <c r="N5" s="14" t="inlineStr">
         <is>
           <t>【收盘前预测·下一开盘日 2026-10-29】
-上证指数：决议落地后中性偏修复 3630~3680；全天 3620~3690；置信度 中低。
-恒生科技：中性偏修复 3790~3860；全天 3770~3880；置信度 中低。
-首要变量：美联储决议（10/29凌晨）、五中全会闭幕公报（29日）、3660/3648得失去、量能能否回升、创业板止跌确认。</t>
+上证指数：平开略偏强 3665~3695；收盘中性偏强 3662~3698；全天 3655~3705；置信度 中低。
+首要变量：美联储10/29凌晨决议（预期按兵不动）、五中全会29日闭幕尾段维稳、3700压力/3655承接、今日反弹量能是否延续、创业板止跌确认。
+恒生科技：平开至小幅高开 3815~3850；收盘中性偏强 3820~3855；全天 3808~3862；置信度 中低。
+首要变量：美联储决议与美债/汇率、南向连续净卖出能否结束、腾讯/美团带动、3900压力/3800防线、隔夜费半与中概传导。
+创业板指：平开至小幅高开 2600~2630；收盘中性 2605~2630；全天 2600~2638；置信度 中低。
+首要变量：今日+3.1%反弹的持续性、2650压力、量能配合、半导体/机器人链止跌。
+恒生指数：平开略偏强 23050~23180；收盘中性 23040~23180；全天 23000~23200；置信度 中低。
+首要变量：美联储决议、南向资金、23160突破、23000关口承接。
+（基准按今日10-28截至14:32实际≈上证3681.66(+0.91%)、恒科3835.18(+0.91%)、创业板2627.25(+3.10%)、恒指23087.83(+0.20%)；预测区间相对10-28收盘遵循≤1%收盘、≤1.5%全天规则；风险提示：若美联储意外加息或“外部映射失效”重现，则整体下修）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: 收盘前精炼 下一开盘日(2026-10-30)预测 · 2026-10-29
</commit_message>
<xml_diff>
--- a/股票预测/股票预测总表.xlsx
+++ b/股票预测/股票预测总表.xlsx
@@ -558,6 +558,7 @@
     <col width="31" customWidth="1" min="11" max="11"/>
     <col width="31" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -976,18 +977,19 @@
           <t>待验证</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
-        <is>
-          <t>【收盘前预测·下一开盘日 2026-10-30】
-上证指数：平开至小幅高开 3683~3705；收盘 3660~3690；全天 3658~3708；置信度 中。
-首要变量：3700关口得失、昨日1.63万亿量能能否延续、五中全会公报（今日午后发布）政策力度、存储链能否接棒光模块、三季报收官雷区。
-创业板指：小幅高开 2640~2658；收盘 2620~2640；全天 2620~2659；置信度 中。
-首要变量：中际旭创/新易盛/天孚通信三剑客（昨日贡献逾五成涨点）是否走弱、2650套牢盘、AI链扩散到存储与被动元件。
-恒生指数：平开略偏弱 23030~23095；收盘 22980~23100；全天 22960~23120；置信度 中低。
-首要变量：金龙指数-1.83%传导、油价102.78美元与12月加息预期、南向资金能否止卖出、22980支撑。
-恒生科技：小幅高开 3845~3875；收盘 3825~3852；全天 3820~3877；置信度 中低。
-首要变量：英伟达-1.17%与美股科技龙头走弱、SK海力士+13.3%对港半导体的正面映射、3825防线与3800关口。
-（基准按10-28收盘：上证3681.47/创业板2634.76/恒指23094.83/恒科3853.72；区间遵循收盘≤1%、全天≤1.5pct规则；风险提示：五中全会公报若表述平淡，午后存在“利好兑现”回落，A股可能高开低走。）</t>
+      <c r="N6" s="14" t="inlineStr">
+        <is>
+          <t>【收盘前预测·下一开盘日 2026-10-30 · 14:15精炼版】
+（基准说明：截至14:15，10-29实际收盘尚未公布（盘中）。本精炼版以早报对10-29的预测收盘为锚≈上证3675/恒科3838/创业板2630/恒指23040；早报对10-29自身判断为“高开冲高回落”，即10-28放量大反弹后进入温和回吐。区间遵循收盘≤1%、全天≤1.5pct规则）
+上证指数：平开至小幅低开 3665~3685；收盘偏弱 3645~3675；全天 3638~3690；置信度 中低。
+首要变量：月终+三季报收官前(10-31截止)的获利了结/避险、3700压力与3655/3640承接、五中全会公报落地后的“利好兑现”风险、量能能否维持1.5万亿、光模块三剑客(中际旭创/新易盛/天孚通信)是否松动。
+恒生科技：平开至小幅低开 3815~3840；收盘偏弱 3805~3835；全天 3793~3848；置信度 中低。
+首要变量：金龙指数-1.83%与美股科技龙头(英伟达-1.17%)传导、南向连续净卖出能否止步、$100+油价对估值压制、3825/3800支撑、五中全会公报对A股情绪的间接带动。
+创业板指：平开至小幅低开 2620~2640；收盘 2605~2635；全天 2600~2638；置信度 中低。
+首要变量：中际旭创/新易盛/天孚通信(昨日贡献逾五成涨点)是否走弱、2650套牢盘、量能配合。
+恒生指数：平开略偏弱 22980~23100；收盘 22960~23100；全天 22940~23120；置信度 中低。
+首要变量：金龙-1.83%传导、南向资金、23160突破/22900承接、油价与美债汇率。
+风险提示：本精炼版为收盘前(14:15)预判，尚未纳入10-29实际收盘；若午后五中全会公报表述平淡或三季报“雷”集中，A股/港股可能进一步下修。AI预测，仅供参考，不构成投资建议。</t>
         </is>
       </c>
     </row>

</xml_diff>